<commit_message>
Upload for Module 3
</commit_message>
<xml_diff>
--- a/Module-3-DataScientist and ML/results/reports/01_data_quality_report.xlsx
+++ b/Module-3-DataScientist and ML/results/reports/01_data_quality_report.xlsx
@@ -839,7 +839,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -886,7 +890,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -933,7 +941,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -980,7 +992,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1027,7 +1043,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1074,7 +1094,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1121,7 +1145,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1168,7 +1196,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1215,7 +1247,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1262,7 +1298,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1309,7 +1349,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1356,7 +1400,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1403,7 +1451,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1450,7 +1502,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1497,7 +1553,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1544,7 +1604,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1591,7 +1655,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1638,7 +1706,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1685,7 +1757,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1732,7 +1808,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1779,7 +1859,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1826,7 +1910,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1873,7 +1961,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1920,7 +2012,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1967,7 +2063,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2014,7 +2114,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2061,7 +2165,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2108,7 +2216,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2155,7 +2267,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2202,7 +2318,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2249,7 +2369,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2296,7 +2420,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2343,7 +2471,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2390,7 +2522,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2437,7 +2573,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2484,7 +2624,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2531,7 +2675,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2578,7 +2726,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2625,7 +2777,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2672,7 +2828,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2719,7 +2879,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2766,7 +2930,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2813,7 +2981,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2860,7 +3032,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2907,7 +3083,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2954,7 +3134,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3001,7 +3185,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3048,7 +3236,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3095,7 +3287,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3142,7 +3338,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3189,7 +3389,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3236,7 +3440,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3283,7 +3491,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3330,7 +3542,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3377,7 +3593,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3424,7 +3644,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3471,7 +3695,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3518,7 +3746,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3565,7 +3797,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3612,7 +3848,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3659,7 +3899,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3706,7 +3950,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3753,7 +4001,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3800,7 +4052,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3847,7 +4103,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3894,7 +4154,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3941,7 +4205,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3988,7 +4256,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4035,7 +4307,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4082,7 +4358,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4129,7 +4409,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4176,7 +4460,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4223,7 +4511,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4270,7 +4562,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4317,7 +4613,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4364,7 +4664,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4411,7 +4715,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4458,7 +4766,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4505,7 +4817,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4552,7 +4868,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4599,7 +4919,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4646,7 +4970,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4693,7 +5021,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4740,7 +5072,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4787,7 +5123,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4834,7 +5174,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4881,7 +5225,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4928,7 +5276,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4975,7 +5327,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5022,7 +5378,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5069,7 +5429,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5116,7 +5480,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5163,7 +5531,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5210,7 +5582,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5257,7 +5633,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5304,7 +5684,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5351,7 +5735,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5398,7 +5786,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5445,7 +5837,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5492,7 +5888,11 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>